<commit_message>
content(members): add Yung-Hsu (Eric) Huang as pre-master's student
Add new member yunghsuhuang: stub member.json + photo.jpg from the
xlsx refresh. Position: Undergraduate (Pre-Master's) Student. About
page and detail fields (interests, links, email) to follow in a
later pass.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contents/members/member-info.xlsx
+++ b/contents/members/member-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jianhern/Desktop/NTU-E3-Center.github.io/contents/members/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B19A4F9-5F74-D941-987C-62215CD3976D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930F1707-E05A-E34C-99C0-3422A4244BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Members" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="201">
   <si>
     <t>WebID</t>
   </si>
@@ -611,6 +611,18 @@
   </si>
   <si>
     <t>黃尹笛</t>
+  </si>
+  <si>
+    <t>Yung-Hsu Huang</t>
+  </si>
+  <si>
+    <t>黃永緒</t>
+  </si>
+  <si>
+    <t>yunghsuhuang</t>
+  </si>
+  <si>
+    <t>MS0</t>
   </si>
 </sst>
 </file>
@@ -950,8 +962,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2093,6 +2108,35 @@
         <v>15</v>
       </c>
     </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>199</v>
+      </c>
+      <c r="B40" t="s">
+        <v>197</v>
+      </c>
+      <c r="C40" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" t="s">
+        <v>198</v>
+      </c>
+      <c r="E40" t="s">
+        <v>65</v>
+      </c>
+      <c r="F40" t="s">
+        <v>116</v>
+      </c>
+      <c r="G40" t="s">
+        <v>47</v>
+      </c>
+      <c r="J40" t="s">
+        <v>200</v>
+      </c>
+      <c r="K40" t="s">
+        <v>118</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(members): add Gloria Kelechi Ukaoma
She was in the roster spreadsheet but invisible on the site: the WebID cell
was blank, and that key is what the pipeline builds a member's content folder
and page URL from, so there was nothing to render.

Adds the WebID, her photo, position (Computer-Aided Engineering Division),
research interests and About text. Also completes her Chinese name — the
sheet had 秀妍 without the 高 surname — and records the name she goes by,
Kelechi, which is what the listing displays.
</commit_message>
<xml_diff>
--- a/contents/members/member-info.xlsx
+++ b/contents/members/member-info.xlsx
@@ -2343,14 +2343,24 @@
       </c>
     </row>
     <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>gloriakelechiukaoma</t>
+        </is>
+      </c>
       <c r="B42" t="inlineStr">
         <is>
           <t>Gloria Kelechi Ukaoma</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Kelechi</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>秀妍</t>
+          <t>高秀妍</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">

</xml_diff>